<commit_message>
feat: implement participant exam submission API, database schema, and supporting backend routes
</commit_message>
<xml_diff>
--- a/outputs/question-import-template/Template_Import_Soal_LMS.xlsx
+++ b/outputs/question-import-template/Template_Import_Soal_LMS.xlsx
@@ -301,7 +301,7 @@
     <t>generated_at</t>
   </si>
   <si>
-    <t>2026-08-29T14:35:50.972Z</t>
+    <t>2026-09-14T08:59:27.474Z</t>
   </si>
   <si>
     <t>Tipe Soal</t>
@@ -1108,7 +1108,7 @@
       <c r="C20" s="13"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="iyezppL464tTCye49c0mDTHA5ERWFI6R0sDd42KbbC2d8+BK5VhI0hqT55ABWgnfcplNDPkhg2XtsjfPrcNzCw==" saltValue="X27Jl8V6Lw/Xnk7/DqAwxg==" spinCount="100000"/>
+  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="baqal4YDz/hRRocK0sqzdaB/8tsvsZc1TqLl1n4PpB5/h4AEh4tuGEUnRsWybs3n3rEzSINzJ6mtzSemLDoK7g==" saltValue="Mx7bw0i3z/f4Nb/e8YwqTw==" spinCount="100000"/>
   <mergeCells count="8">
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A2:C2"/>
@@ -33542,7 +33542,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="EvaarMI3SUyUwd6W7RuV4dVkdSCfB1y8nTmodJsq5sPFjcFFu445wpPbIX0fZYz31SOS0ffPhstEkOGbrmg6TA==" saltValue="RnaJ6OkCmSXJqzKMoHaHtg==" spinCount="100000"/>
+  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="d6QvU0z96U8KNX6f/7erITdtu0vs7f33K7vHN/e4jv8McHY554wWg9r9aBk8HxAo73iUU1iSN716YfY/88qogA==" saltValue="IzwgoESdpFpfMCB6Me0kjw==" spinCount="100000"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
@@ -33613,7 +33613,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="c7v44Ok/qBcVfPqJp0pcrTJZNWe7zAyHMqa4H8nTz02qBJ9NMdW5IKO7VD6LzUHChtJk7Obr1plHFcRmUAOS1Q==" saltValue="MN1jDunmVqa1ueIUrxymYg==" spinCount="100000"/>
+  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="qEfDG4qSG91vfV+olalTkcV12AGA2oxwT/RYklHjhi+XaY1ML97bsjKvcdr9bJlqJX2MzuAX8XeGwDRNlIHvaA==" saltValue="iLFUDWnAgXW5nirb5NM1bQ==" spinCount="100000"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -33740,7 +33740,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="HNIlJXA0a7Ngqo6Pzef/wvxW7KXSnL3XZfu+wxodbUWHRPRynHEGlspRTAWHFF46qWYul0mWzrpiyq65lcnFMA==" saltValue="VFGLjfIU209LwIqxWeC5iw==" spinCount="100000"/>
+  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="cXVSXlPPybQTFsgXk1f3pujt/wRL0JpgvZaMsdPXSFZz+C+mym6KED9fsWricYsLoWTs9UqnNumz69z0lJnuug==" saltValue="n1bn1BL6ayA3IXwYZIvRpQ==" spinCount="100000"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>

<commit_message>
Refine LMS features and user workflows
</commit_message>
<xml_diff>
--- a/outputs/question-import-template/Template_Import_Soal_LMS.xlsx
+++ b/outputs/question-import-template/Template_Import_Soal_LMS.xlsx
@@ -301,7 +301,7 @@
     <t>generated_at</t>
   </si>
   <si>
-    <t>2026-09-14T08:59:27.474Z</t>
+    <t>2026-09-18T04:07:49.686Z</t>
   </si>
   <si>
     <t>Tipe Soal</t>
@@ -1108,7 +1108,7 @@
       <c r="C20" s="13"/>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="baqal4YDz/hRRocK0sqzdaB/8tsvsZc1TqLl1n4PpB5/h4AEh4tuGEUnRsWybs3n3rEzSINzJ6mtzSemLDoK7g==" saltValue="Mx7bw0i3z/f4Nb/e8YwqTw==" spinCount="100000"/>
+  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="ycPD5em+DKHXh4oY2iPPOwSXqa1F9njaG2CEUhab9XTnNDLr/DwZjakDcCnydblJrA4bXflQGEeisWwx8WJ4Lw==" saltValue="JDqRZBL7/deLToEhWAedGw==" spinCount="100000"/>
   <mergeCells count="8">
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A2:C2"/>
@@ -33542,7 +33542,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="d6QvU0z96U8KNX6f/7erITdtu0vs7f33K7vHN/e4jv8McHY554wWg9r9aBk8HxAo73iUU1iSN716YfY/88qogA==" saltValue="IzwgoESdpFpfMCB6Me0kjw==" spinCount="100000"/>
+  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="LitlMr33I7d5nQV1Z0jjneLRoFT3dtzP0PktPMVA3PNzyu0AfNJ+LxiauAR21I/SWVtTQ45mb/7+ZsZjLf4a/g==" saltValue="bT7IF9jL0DAqHiOd4zEAbQ==" spinCount="100000"/>
   <mergeCells count="1">
     <mergeCell ref="A1:F1"/>
   </mergeCells>
@@ -33613,7 +33613,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="qEfDG4qSG91vfV+olalTkcV12AGA2oxwT/RYklHjhi+XaY1ML97bsjKvcdr9bJlqJX2MzuAX8XeGwDRNlIHvaA==" saltValue="iLFUDWnAgXW5nirb5NM1bQ==" spinCount="100000"/>
+  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="4Ff+YsYEn4RaSc9hlV9krt3o4MG3Rrhy/wyylP6XgGzh7+Cs5bHvgEdv6qJBW71J4a6saYvttZoTBW8tKr4kBA==" saltValue="Z5/r1U0Ls36t6rI2Vf/1+g==" spinCount="100000"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -33740,7 +33740,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="cXVSXlPPybQTFsgXk1f3pujt/wRL0JpgvZaMsdPXSFZz+C+mym6KED9fsWricYsLoWTs9UqnNumz69z0lJnuug==" saltValue="n1bn1BL6ayA3IXwYZIvRpQ==" spinCount="100000"/>
+  <sheetProtection sheet="1" algorithmName="SHA-512" hashValue="Edhz1s8RWi4riUbA1T4+p4TBvZmaz9b76fh9eh5PfVzJKfIZ3GFEkR69DqfmES9hEY4f4F8pHrNaGXpdMMKv8g==" saltValue="J27klCueGra05CdhKyWaKQ==" spinCount="100000"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>